<commit_message>
se agrega unitario por exportadora y especie
</commit_message>
<xml_diff>
--- a/uploads/ultima_estimacion.xlsx
+++ b/uploads/ultima_estimacion.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/740e28deca2ef4c4/Almahue/Gestion/Facturacion Planta/Temp2026/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\172.20.20.5\Airflow\dags\data\bd\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{94707426-6652-4A9D-B3E6-0CF07E15C5BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9E9615BD-FFE8-4A04-B78E-2154BC376527}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BCCE9F7-8547-42FA-ACF1-47CB778F38BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="555" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BD" sheetId="1" r:id="rId1"/>

</xml_diff>